<commit_message>
target_space ground-truth labels v1: 19 papers, single-rater author-labelled, protocol v1.2
</commit_message>
<xml_diff>
--- a/ground_truth/target_space_labels_v1.xlsx
+++ b/ground_truth/target_space_labels_v1.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19880" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Start here" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,18 +11,64 @@
     <sheet name="Labels" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Times"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color rgb="FFD3D7DE"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color rgb="FF9BE963"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
@@ -37,9 +82,6 @@
     <font>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
-    </font>
-    <font>
-      <i val="1"/>
     </font>
   </fonts>
   <fills count="6">
@@ -70,10 +112,36 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -82,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -103,21 +171,42 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -480,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B20"/>
+  <dimension ref="B2:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -488,21 +577,21 @@
   </cols>
   <sheetData>
     <row r="2">
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>fMRI target_space labeling — 18 papers, ~15 min each</t>
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>fMRI target_space labeling — 19 papers, ~15 min each</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Thank you for doing this. You are establishing an independent 'answer key' for ONE field — the VOLUMETRIC normalization target of the functional pipeline (spatial_normalization.target_space) — against which an automated extraction tool will be scored. Your labels are compared to a second labeler's to measure agreement (Cohen's kappa; deferred, conditional on publication), so please work independently.</t>
+          <t>Independent 'answer key' for ONE field — the VOLUMETRIC normalization target of the functional pipeline (spatial_normalization.target_space). Label what the PAPER states, not what a file/citation resolves to beyond established identity. Protocol v1.2 (docs/ground-truth-protocol-target_space.md).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>The one rule that matters most</t>
         </is>
@@ -511,12 +600,12 @@
     <row r="7">
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Label the VOLUMETRIC target the PAPER states — not what you know a file or citation resolves to beyond ESTABLISHED IDENTITY. 'MNI' stays family_specified even though you may suspect NLin6Asym; only a named variant or a specific template FILE (oconnor: FSL's MNI152T1_2mm_brain.nii.gz) earns canonical. Writing the resolved variant for a bare 'MNI' would score the tool's job as if it were the paper's.</t>
+          <t>Record where the functional TIMESERIES ends up volumetrically (CALL 7). Normalization of derived statistical maps, or a surface projection, does not set target_space. A named volumetric template the timeseries reaches wins even if data are later projected to a surface (weber); a timeseries that reaches no volumetric template is native_volume (binder, chen).</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>Surface templates are a DIFFERENT axis — do NOT label them here</t>
         </is>
@@ -525,12 +614,12 @@
     <row r="10">
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>fsaverage, fsaverage5, Conte69, fsLR/fs_LR and other SURFACE templates are NOT target_space values — they belong to a separate field (target_surface). target_space records ONLY the volumetric stereotactic target. A surface-based paper that also states a volumetric target is labeled on that volumetric target; a purely-surface paper with no volumetric target is 'absent' here. (See CALL 1 in the Glossary.)</t>
+          <t>fsaverage/fsaverage5, Conte69, fsLR are SURFACE templates (target_surface), never target_space (CALL 1). chen's only 'MNI' is the surface template's frame via sphere registration → native_volume.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="18" t="inlineStr">
         <is>
           <t>What to do</t>
         </is>
@@ -539,49 +628,21 @@
     <row r="13">
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>1.  Go to the 'Labels' tab. There is one row per paper (18 papers).</t>
+          <t>1.  Go to 'Labels'. One row per paper (19). 2. Read each paper in FULL. 3. Fill target_space_state (dropdown), Value, Supporting quote; Notes optional. 4. Two YELLOW example rows show the format.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2.  For each paper, read it in FULL (methods, figure captions, data-availability, and supplement if you have it) — not just the methods sentence. Specific template files often live outside the one sentence a tool would quote.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>3.  Fill the GREEN columns: target_space_state (dropdown), Value, Supporting quote. Notes is optional.</t>
+          <t>5.  Label blind — do NOT look at extractor output first. 6. A composed transform chain stated end-to-end and terminating in a named template specifies that template (CALL 6). 7. If a paper fits none of the six states, note why rather than forcing it.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>4.  The two YELLOW example rows at the top are filled in for you — copy their format.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>5.  Do NOT look at any extractor / tool output before deciding. The denominator must be independent of the tool being measured.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>6.  If a paper doesn't fit the six states, write your reasoning in Notes rather than forcing a label — amend the protocol, bump the version, re-commit, THEN label it. That's useful signal, not a failure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Full definitions and every state option are on the 'Glossary' tab. You should not need any other document.</t>
+          <t>Full definitions, the six states, and CALLs 1–7 are on the 'Glossary' tab.</t>
         </is>
       </c>
     </row>
@@ -596,7 +657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C19"/>
+  <dimension ref="B2:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -605,7 +666,7 @@
   </cols>
   <sheetData>
     <row r="2">
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="19" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
@@ -617,14 +678,14 @@
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="18" t="inlineStr">
         <is>
           <t>target_space_state</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Pick ONE (dropdown). The completeness with which the paper specified its VOLUMETRIC stereotactic target:</t>
+          <t>Pick ONE (dropdown). Completeness of the VOLUMETRIC stereotactic target:</t>
         </is>
       </c>
     </row>
@@ -636,7 +697,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>The paper named a SPECIFIC, RESOLVABLE template: a variant identifier (MNI152NLin6Asym, MNI152NLin2009cAsym), OR a specific template FILE that resolves to one by established identity (oconnor: FSL's MNI152T1_2mm_brain.nii.gz -&gt; MNI152NLin6Asym; FSL ships NLin6Asym), OR Talairach with its atlas.</t>
+          <t>A specific, resolvable template: a variant identifier (MNI152NLin6Asym / MNI152NLin2009cAsym), OR a specific template FILE that resolves by established identity (oconnor: FSL's MNI152T1_2mm_brain.nii.gz), OR Talairach with its atlas.</t>
         </is>
       </c>
     </row>
@@ -648,7 +709,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>The paper named the MNI family (or a tool-generic MNI reference) WITHOUT a resolvable variant: 'MNI', 'MNI152', 'MNI standard space', 'SPM's MNI template', 'MNI-152 12-dof linear'. Real, era-standard specification — NOT a failure, a completeness tier. When unsure whether a reference resolves to ONE template, it is family_specified (canonical is the stricter claim).</t>
+          <t>Named a TEMPLATE — a family term, tool-generic reference, or tool-shipped template — WITHOUT a resolvable variant: 'MNI', 'MNI152', 'SPM MNI template' (wheaton), 'an EPI template' (gordon). Each names a template ARTIFACT/family that EXISTS as a file. A bare 'atlas'/'standard space' gesture names no artifact → absent, NOT family_specified. (CALL 2/3)</t>
         </is>
       </c>
     </row>
@@ -660,7 +721,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>The paper normalized to a template CONSTRUCTED for this study (developmental/cohort/precision; mueller: subject-specific template via ANTs multivariate template construction). A specified methodological choice, dataset-bound.</t>
+          <t>Normalized to a template CONSTRUCTED for this study (mueller: ANTs multivariate template construction; ciric: study-specific PNC template reached via a stated two-leg chain — CALL 6).</t>
         </is>
       </c>
     </row>
@@ -672,7 +733,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>No volumetric normalization; functional data kept in each subject's own volumetric space — a stated choice ('no normalization' is itself specification). Distinct from study_specific (which DOES normalize, to a constructed template) and from absent (which reports nothing). NB: a paper that resamples into an even-unnamed common atlas grid is NOT native_volume (see CALL 4).</t>
+          <t>The functional TIMESERIES receives NO volumetric template. Two forms: explicitly kept native (CALL 3), OR terminal volumetric state identifiable from an enumerated step sequence AND native — exits to surface (chen, CALL 7b) or only derived maps normalized (binder, CALL 7a). NB: resampling into an unnamed atlas GRID is NOT native_volume → deferred (poldrack, CALL 4).</t>
         </is>
       </c>
     </row>
@@ -684,7 +745,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>The paper names no volumetric target itself but attributes its pipeline (hence the target) to a cited work or named-by-provenance pipeline, so the target plausibly lives in that citation — identity UNRESOLVED (poldrack: 'a pipeline developed at Washington University, St Louis[45]'). Distinct from absent (nothing anywhere) and from canonical/family_specified (which need an in-hand named target). Mirrors base_pipeline's DEFERRED_TO_CITATION. Assert no specific template; resolving the citation is the downstream citation-resolver's job.</t>
+          <t>No volumetric target named in-paper, but the pipeline (hence target) is attributed to a cited/provenance-named work — plausibly in that citation, identity UNRESOLVED (poldrack: 'a pipeline developed at Washington University, St Louis[45]'). Mirrors base_pipeline DEFERRED_TO_CITATION. Assert no specific template.</t>
         </is>
       </c>
     </row>
@@ -696,115 +757,151 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>No reconstructable volumetric target at all AND no deferral: 'atlas space' / 'standard space' with no template named, or silence. Contrast deferred (target named only in a cited work). A resolution (3 mm) or d.o.f. without a template does NOT upgrade this — that is a separate field (resolution_mm).</t>
+          <t>No reconstructable volumetric target AND no deferral: a bare coordinate-SPACE or transformation naming no template artifact — 'atlas', 'atlas space', 'atlas transformation' (power), 'standard space' — or silence. 'Atlas' is a gesture, not a named template.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="18" t="inlineStr">
         <is>
           <t>Value (verbatim)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>The volumetric target as the paper WRITES it, verbatim: 'MNI', 'FSL's MNI152T1_2mm_brain.nii.gz', 'MNI-152 template (12-dof linear)', 'atlas space'. For absent, leave blank or note the gesture ('atlas space').</t>
+          <t>The verbatim target TERM when the paper names one (power: 'atlas'). BLANK when it does not (braun, viduarre, binder, chen). The Value column holds ONLY the verbatim target term — the adjudication goes in Notes (so a machine-read CSV has one meaning per column).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="18" t="inlineStr">
         <is>
           <t>Supporting quote (verbatim)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>The exact sentence stating the volumetric target. Copy it VERBATIM (it gets checked against the paper text). Required for every non-absent label; for canonical the quote must contain the specific variant/file. For absent, note the gesture or that nothing was stated.</t>
+          <t>The exact sentence(s), copied VERBATIM including any source typos (checked against the paper). Required for every non-absent label; for canonical the quote must contain the specific variant/file; for a composed chain (CALL 6) quote EVERY leg.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="18" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Hard calls, open questions, or what a citation resolves to. Optional but valued.</t>
+          <t>The adjudication, hard calls, the composition (CALL 6), open lineage (wheaton/gordon), or what a citation resolves to.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>The hard lines (from the protocol)</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>See docs/ground-truth-protocol-target_space.md for the full text.</t>
+      <c r="B14" s="20" t="inlineStr">
+        <is>
+          <t>The hard lines (protocol v1.2)</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>See docs/ground-truth-protocol-target_space.md for full text.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>CALL 1 (ratified)</t>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>CALL 1</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>target_space is VOLUMETRIC ONLY. Surface templates (fsaverage5, Conte69, fsLR) route to target_surface, a separate axis — verified at HEAD to be genuinely EXTRACTED, so it is a real field, not schema-only. chen ('MNI' + fsaverage5) and weber ('MNI152' + Conte69) are family_specified HERE on their volumetric 'MNI'; their surface template is out of scope for this field.</t>
+          <t>target_space is VOLUMETRIC ONLY; surface templates route to target_surface (a distinct, genuinely-extracted field). chen's MNI is the surface frame (sphere registration), not volumetric.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>CALL 2 (ratified)</t>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>CALL 2</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>canonical vs family_specified turns on RESOLVABILITY to a specific variant/file, not how official the name sounds. wheaton 'SPM MNI template' -&gt; family_specified for now (OPEN: SPM lineage is variant-ambiguous; do not promote to canonical without verifying which template SPM shipped, possibly needing a linear-MNI152 enum value). derosa 'MNI-152, 12-dof linear' -&gt; family_specified (names family + d.o.f., not a variant/file).</t>
+          <t>canonical vs family_specified = resolvability to a specific variant/file, not how official the name sounds. wheaton 'SPM MNI template' → family_specified for now (OPEN lineage question).</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>CALL 3 (ratified)</t>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>CALL 3</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>The low-specification boundary: family named -&gt; family_specified; no template but native space stated -&gt; native_volume; no template and no native statement -&gt; absent. power/poldrack 'atlas space' -&gt; absent ('atlas space' names no template; the 3 mm is resolution_mm, not the space).</t>
+          <t>family/native/deferred/absent boundary. ARTIFACT vs SPACE: a named template artifact/family (MNI, EPI template) → family_specified; a bare 'atlas'/'standard space' with no artifact → absent (power). A resolution/d.o.f. without a template does not upgrade absent.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>CALL 4 (RATIFIED v1.1 — narrow form)</t>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>CALL 4</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>DUAL-AXIS: completeness is reported PER AXIS, and a paper is exempt from a VOLUMETRIC reporting-gap ONLY under the conjunction (i) volumetric target unnamed in-paper AND (ii) volumetric analysis units individually-defined (e.g. CIFTI grayordinates + subcortical regions from the subject's OWN FreeSurfer segmentation). NEVER 'surface/CIFTI paper =&gt; volumetrically exempt'. A paper that NAMES a volumetric template is family_specified and gets NO exemption (chen 'MNI', weber 'MNI152' -&gt; family_specified, no credit-by-substitution from their surface). Consequence: the headline is TWO distributions (volumetric + surface) plus a joint statement, papers in both — not one number. poldrack: volumetric deferred, surface canonical 32k fs_LR, exempt from a volumetric reporting failure (its volumetric units are individually-defined; honest caveat: the BOLD IS resampled into the unnamed atlas grid as a registration substrate).</t>
+          <t>DUAL-AXIS: completeness reported PER AXIS. A paper is exempt from a volumetric reporting-gap ONLY under the conjunction [volumetric target unnamed in-paper AND volumetric units individually-defined]. Headline = two distributions + a joint statement, papers in both.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>CALL 5 (RESOLVED v1.1 — Option A)</t>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>CALL 5</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>'deferred' is ADDED as the sixth state (now in the dropdown). absent (nothing reconstructable anywhere) and deferred (named only in a cited work) are different reproducibility facts — the spine of the provenance model AESPA is built on; a vocabulary narrower than base_pipeline's would be an inconsistency to explain. poldrack's v1 volumetric 'absent' is SUPERSEDED to 'deferred' (its pipeline is attributed by provenance to a cited WashU pipeline; base_pipeline labels the same construct DEFERRED, so 'absent' here would contradict a committed protocol). deferred asserts no specific template — do not resolve it.</t>
+          <t>'deferred' is the sixth state (Option A). poldrack volumetric superseded absent → deferred (provenance-named cited pipeline), consistent with base_pipeline's DEFERRED.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>CALL 6</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>A composed transform chain stated end-to-end in-paper and terminating in a NAMED template specifies that template (ciric → study_specific via structural-leg + BBR). Complete chain to an UNNAMED terminal → deferred (poldrack). Every leg must be in the text; Notes records the composition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>CALL 7</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>target_space = terminal volumetric state of the functional TIMESERIES. (a) normalizing derived statistical maps does not set it (binder → native_volume); (b) a timeseries that exits to the surface axis with no stated volumetric target is native_volume (chen). Reconciles with CALL 3: native_volume = explicit native statement OR identifiable native terminal state (not an atlas grid).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>Recording convention</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Value = the verbatim target term when named, blank otherwise; Notes carries the adjudication. native_volume is evidenced by a positive quote plus the absence of any volumetric-normalization step (stated OR evident from the enumerated pipeline).</t>
         </is>
       </c>
     </row>
@@ -820,7 +917,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -829,7 +926,7 @@
     <col width="34" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="16" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Paper</t>
@@ -856,260 +953,564 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+    <row r="2" ht="160" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>oconnor_2017 (EXAMPLE)</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>canonical</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="9" t="inlineStr">
         <is>
           <t>FSL's MNI152T1_2mm_brain.nii.gz</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="9" t="inlineStr">
         <is>
           <t>A non-rigid registration between MPRAGE images and a 2-mm MNI brain-only template (FSL's MNI152T1_2mm_brain.nii.gz, [59]) was calculated using ANTs [60].</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="9" t="inlineStr">
         <is>
           <t>Names a SPECIFIC resolvable FSL template FILE -&gt; canonical (FSL ships MNI152NLin6Asym; verified vs FSL docs / TemplateFlow / Lead-DBS). NB: the extractor flattens this to 'MNI' (family_specified) — the one extraction miss on this corpus (see docs/findings/extraction-specificity-flattening.md). Label what the PAPER stated. (Example row — do not edit.)</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+    <row r="3" ht="80" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>mueller_2021 (EXAMPLE)</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>study_specific</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>subject-specific anatomical template (ANTs multivariate template construction)</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>All scans were then registered to a subject-specific anatomical template created using Advanced Normalization Tools (ANTs) multivariate template construction.</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>Normalized to a template CONSTRUCTED for this study -&gt; study_specific, NOT family_specified (no MNI family named) and NOT absent (a template WAS built). (Example row — do not edit.)</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+    <row r="4" ht="224" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>agtzidis_2020</t>
         </is>
       </c>
-      <c r="B4" s="10" t="n"/>
-      <c r="C4" s="10" t="n"/>
-      <c r="D4" s="10" t="n"/>
-      <c r="E4" s="10" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>family_specified</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>MNI</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>coregistering them to the anatomical T1 scan, normalizing
+them to the MNI template,</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>Note for surface - results in surface but not analyses: "Results
+The presented functional group results of this section were mapped to
+the three-dimensional cortical template of the“Population-Average,
+Landmark- and Surface-based” Atlas (PALS) (Van Essen, 2005) with the
+metric-enclosing-voxel algorithm in Caret (version 5.65) (Van Essen
+et al., 2001). When needed, the provided coordinates are reported in the
+Montreal Neurological Institute (MNI) coordinate system."</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>braun_2015</t>
         </is>
       </c>
-      <c r="B5" s="10" t="n"/>
-      <c r="C5" s="10" t="n"/>
-      <c r="D5" s="10" t="n"/>
-      <c r="E5" s="10" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="n"/>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Data
+were preprocessed according to standard protocols as previously described in
+refs. 47 and 48. After preprocessing, the mean time series in 5-mm spheres
+around coordinates defined by ref. 36 were extracted.</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="n"/>
+    </row>
+    <row r="6" ht="409.6" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>chen_2015</t>
         </is>
       </c>
-      <c r="B6" s="10" t="n"/>
-      <c r="C6" s="10" t="n"/>
-      <c r="D6" s="10" t="n"/>
-      <c r="E6" s="10" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>native_volume</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>With such information, individual pial (GM/CSF boundary) and white (GM/WM boundary) surfaces were reconstructed and spatially normalized to match a group-level standard template surface in the Montreal Neurological Institute (MNI) space via a sphere registration [49, 54, 55]. The subsequent CCS functional pipeline discarded the first 5 EPI volumes (10 seconds), removed and interpolated temporal spikes (see instructions in [56, 57] regarding in-scanner head motion), corrected acquisition timing among image slices and head motion among image volumes and normalized the 4D global mean intensity to 10,000. White surfaces were then employed by a boundary-based registration (BBR) algorithm to match spatial correspondences between individual functional images to anatomical images [58]. To further eliminate the effect of head motion and physiological noises during the rfMRI scanning session, we regressed out the estimated Friston’s 24-parameter motion curves [37] and nuisance signals measured as WM and CSF mean time series [59] from individual rfMRI time series. Linear and quadratic trends were also regressed out from the rfMRI data by multiple linear regressions. Finally, the data were projected onto the fsaverage surface grid (average inter-vertex distance = 1 mm) and
+down-sampled to the fsaverge5 surface grid (average inter-vertex distance = 4 mm) for subse-quent rfMRI computation. Participant-level rfMRI Metrics Derivation
+The overall analytic strategy is presented in Fig 1. The above CCS pipeline preprocessed all individual rfMRI images (Fig 1A) and projected individual rfMRI time series onto a uniform cortical surface grid (fsaverge5) based upon the brain tissue classification (Fig 1B and 1C). As a proof of concept, an individual-level functional connectome can be modeled as a graph or net-
+work with vertices as nodes and pair-nodes dependency as edges (Fig 1D).</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>Volumetric target not stated in either stream. Anatomical normalization is surface-based only ("via a sphere registration"); the functional stream terminates at the fsaverage5 surface after BBR to subject anatomy. The MNI reference is the surface template's coordinate frame → target_surface per CALL 1, not target_space. Per CALL 7(b): timeseries exits to the surface axis with no volumetric template → native_volume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="176" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>ciric_2017</t>
         </is>
       </c>
-      <c r="B7" s="10" t="n"/>
-      <c r="C7" s="10" t="n"/>
-      <c r="D7" s="10" t="n"/>
-      <c r="E7" s="10" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>study_specific</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>subsample ANTs study-specific template</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>A study-specific template was generated from a sample of 120 PNC subjects balanced across sex, race, and age bins using the build Template Parallel procedure in ANTs (Avants et al., 2011a). Study-specific tissue priors were created using a multi-atlas segmentation procedure (Wang et al., 2014). Next, each subject's high-resolution structural image was processed using the ANTs Cortical Thickness Pipeline (Tustison et al., 2014). Following
+bias field correction (Tustison et al., 2010), each structural image was diffeomorphically registered to the study-specific PNC template using the top-performing SyN deformation (Klein et al., 2009). Study-specific tissue priors were used to guide brain extraction and segmentation of the subject's structural image (Avants et al., 2011b).</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>target reached by composition (func→struct BBR; struct→PNC template SyN), no single stated func→template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>cole_2013</t>
         </is>
       </c>
-      <c r="B8" s="10" t="n"/>
-      <c r="C8" s="10" t="n"/>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="10" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>family_specified</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Talairach</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>normalization to a Talairach template</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="n"/>
+    </row>
+    <row r="9" ht="64" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>derosa_2025</t>
         </is>
       </c>
-      <c r="B9" s="10" t="n"/>
-      <c r="C9" s="10" t="n"/>
-      <c r="D9" s="10" t="n"/>
-      <c r="E9" s="10" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>family_specified</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>MNI-152 template</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Individual subject EPI images were registered to that
+subject’s MPRAGE structural image via linear Boundary-Based Registration
+and then registered to the MNI-152 template via 12 degrees of
+freedom linear transformation.</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="n"/>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>gordon_2014</t>
         </is>
       </c>
-      <c r="B10" s="10" t="n"/>
-      <c r="C10" s="10" t="n"/>
-      <c r="D10" s="10" t="n"/>
-      <c r="E10" s="10" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>family_specified</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>epi template</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Images were then slice-time corrected, normalized to an
+EPI template, and smoothed using a Gaussian kernel with
+full-width at half-maximum (FWHM) of 8 mm.</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>gordon named "an EPI template" (a tool-shipped template artifact) -&gt; family_specified per the broadened CALL 3 definition. CAVEAT: the referent (SPM's stock EPI template) and the stereotactic space it occupies are BOTH unverified -- same open lineage question as wheaton's "SPM MNI template" under CALL 2. Do not assert SPM-EPI-is-MNI; the paper does not state it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="208" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>liu_2005</t>
         </is>
       </c>
-      <c r="B11" s="10" t="n"/>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="10" t="n"/>
-      <c r="E11" s="10" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>family_specified</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Talairach</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Each participant’s high-resolution anatomic volume was trans- formed into Talairach space (Talairach and Tournoux, 1988), after which an automated segmentation procedure was applied to ob- tain a surface reconstruction of the white-gray matter boundary. The surface was further inflated to reveal the sulci/gyri pattern. All analyses were performed on this inflated representation of the cor-
+tical sheet. Preprocessing of functional data included slice time
+correction, motion correction, linear trend removal, and temporal
+high-pass filtering (three cycles per scan) to remove slow drifts in
+the fMRI signal. Given the block design, no slice time correction
+was applied to data from the localizer scan. The 2D functional data
+were then aligned with the high-resolution anatomic volume and
+transformed into 3D data in the Talairach space </t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="n"/>
+    </row>
+    <row r="12" ht="160" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>liu_2013</t>
         </is>
       </c>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="10" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>family_specified</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>152-brain Montreal Neurological Institute (MNI)</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>The fMRI data was first co-registered to the high-resolution
+anatomical (T1-weighted) images acquired from the same sub-
+ject and then normalized to the 152-brain Montreal Neurological Institute (MNI) normalized space. Here, as departure from
+the original FCP scripts, the registration between the func-
+tional and anatomical images was implemented using the
+“align_epi_anat.py” program (Saad et al., 2009) in AFNI, which
+was found to provide a better registration in the superior-inferior
+direction. The pre-processed fMRI data were then resampled at
+the 3 × 3 × 3 mm3 resolution of the MNI normalized brain space.</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="n"/>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>mueller_2021</t>
         </is>
       </c>
-      <c r="B13" s="10" t="n"/>
-      <c r="C13" s="10" t="n"/>
-      <c r="D13" s="10" t="n"/>
-      <c r="E13" s="10" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>study_specific</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>subject-specific anatomical template (ANTs multivariate template construction)</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>All scans were then registered to a subject-specific anatomical template created using Advanced Normalization Tools (ANTs)
+multivariate template construction.</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="n"/>
+    </row>
+    <row r="14" ht="160" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>oconnor_2017</t>
         </is>
       </c>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>canonical</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>FSL's MNI152T1_2mm_brain.nii.gz</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>A non-rigid registration between MPRAGE images and a 2-mm MNI brain-only template (FSL's MNI152T1_2mm_brain.nii.gz, [59]) was calculated using ANTs [60].</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Names a SPECIFIC resolvable FSL template FILE -&gt; canonical (FSL ships MNI152NLin6Asym; verified vs FSL docs / TemplateFlow / Lead-DBS). NB: the extractor flattens this to 'MNI' (family_specified) — the one extraction miss on this corpus (see docs/findings/extraction-specificity-flattening.md). Label what the PAPER stated. (Example row — do not edit.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="208" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>poldrack_2015</t>
         </is>
       </c>
-      <c r="B15" s="10" t="n"/>
-      <c r="C15" s="10" t="n"/>
-      <c r="D15" s="10" t="n"/>
-      <c r="E15" s="10" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>atlas</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>fMRI preprocessing. All fMRI data were preprocessed according to a pipeline developed at Washington University, St Louis45. Data were realigned to correct for head motion and normalized to a mode of 1,000 (one multiplicative constant applied to all voxels and all frames). Each session was registered to a single session that had previously been registered to the mean T1-weighted structural image and
+an atlas. The session-to-atlas transform was inverted and applied to the mean field map so that the distortion correction could be applied in each session’s space. The undistorted data were then re-registered to the atlas space. The transforms for head motion correction and affine registration to atlas space were combined with the field-map-based distortion correction to resample the data from the original session space to the undistorted 3-mm isotropic atlas space in a single step using FSL’s applywarp tool46.</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="n"/>
+    </row>
+    <row r="16" ht="64" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>power_2014</t>
         </is>
       </c>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>absent</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>atlas</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Atlas transformation of the functional data was computed for each individual via the T2-weighted and MP-RAGE scans. Each run was then resampled in atlas space on an isotropic 3 mm grid combining realignment and atlas transformation in a single interpolation (Shulman et al., 2010).</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="n"/>
+    </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>tang_2025</t>
         </is>
       </c>
-      <c r="B17" s="10" t="n"/>
-      <c r="C17" s="10" t="n"/>
-      <c r="D17" s="10" t="n"/>
-      <c r="E17" s="10" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>family_specified</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>MNI standard space</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>then normalizing to MNI standard space and resampling to 3 × 3 × 3 mm3 voxels;</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="n"/>
+    </row>
+    <row r="18" ht="64" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>vanderwal_2016</t>
         </is>
       </c>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>family_specified</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Montreal Neurological Institute (MNI) space</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>Data processing. Standard data preprocessing was performed using the Con-
+figurable Pipeline for Analysis of Connectomes (C-PAC) including motion re-
+alignment and transformation into Montreal Neurological Institute (MNI) space using Advanced Normalization Tools (Avants et al., 2008).</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="n"/>
+    </row>
+    <row r="19" ht="192" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>viduarre_2017</t>
         </is>
       </c>
-      <c r="B19" s="10" t="n"/>
-      <c r="C19" s="10" t="n"/>
-      <c r="D19" s="10" t="n"/>
-      <c r="E19" s="10" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="n"/>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data and Preprocessing. We used resting-state fMRI data from Ν= 820 subjects from the HCP, which provides the required ethics and consent needed for study and dissemination, such that no further institutional review board (IRB) approval is required. These are all subjects with complete resting fMRI data from the
+900-subject public data release, all healthy adults (aged 22–35 y, 453 females) scanned on a 3-T Siemens connectome-Skyra. For each subject, four 15-min runs of fMRI time series data with a temporal resolution of 0.73 s and a spatial res-olution of 2-mm isotropic were available. The preprocessing pipeline followed the technique of Smith et al. (18, 39), and thus will be described only briefly here. Spatial preprocessing was applied using the procedure described by Glasser et al. 40. </t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="n"/>
+    </row>
+    <row r="20" ht="96" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>weber_2024</t>
         </is>
       </c>
-      <c r="B20" s="10" t="n"/>
-      <c r="C20" s="10" t="n"/>
-      <c r="D20" s="10" t="n"/>
-      <c r="E20" s="10" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>family_specified</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>MNI152 space</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>Both T1w and rs-fMRI data were
+linearly co-registered and mapped to MNI152 space.
+Functional imaging data were mapped to correspond-
+ing mid-thickness surfaces. We resampled data to the
+Conte69 surface template [79] via Workbench [78] with
+10,242 surface points (vertices) per hemisphere.</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="n"/>
+    </row>
+    <row r="21" ht="112" customHeight="1">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>wheaton_2004</t>
         </is>
       </c>
-      <c r="B21" s="10" t="n"/>
-      <c r="C21" s="10" t="n"/>
-      <c r="D21" s="10" t="n"/>
-      <c r="E21" s="10" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>family_specified</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>SPM MNI template</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>Data were analyzed using SPM99. Following motion correc-
+tion and slice timing adjustment, each subject’s EPI data were
+spatially normalized to the SPM MNI template and smoothed with
+a 7-mm full width at half maximum (FWHM) isometric Gaussian
+kernel.</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>Additional analyses in native space: "For each subject, motion-corrected, slice timing adjusted EPI data that were not spatially normalized were aligned to their high-resolution T1 SPGR anatomical images and smoothed with a 4 4 7 mm FWHM Gaussian kernel."</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="128" customHeight="1">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>binder_1999</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>native_volume</t>
+        </is>
+      </c>
+      <c r="D22" s="14" t="inlineStr">
+        <is>
+          <t>All EPI images were spatially coregistered using an itera-
+tive procedure that minimizes variance in voxel intensity
+differences between images (Cox, 1996b).</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="inlineStr">
+        <is>
+          <t>Individual anatomical (SPGR) scans and SPMs were
+then projected into the standard stereotaxic space of
+Talairach and Tournoux (1988), using the MCW-AFNI
+software package (Cox, 1996a). - statmaps transformed to talairach space
+native (within-subject coregistration only) — volumetric target state, moved here from Value per the recording convention (Value column = verbatim target term only).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="224" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>GREEN = fill these in.   YELLOW = examples (don't edit).   VOLUMETRIC target only — surface templates (fsaverage/Conte69/fsLR) are a separate axis, not labeled here (CALL 1).   Label what the paper STATES, not what a citation/file resolves to beyond established identity.</t>
         </is>
@@ -1117,7 +1518,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B4:B21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B4:B22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"canonical,family_specified,study_specific,native_volume,deferred,absent"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>